<commit_message>
chore(templates): actualiza plantilla OT-MUESTRAS-Geofal.xlsx
</commit_message>
<xml_diff>
--- a/app/templates/OT/OT-MUESTRAS/OT-MUESTRAS-Geofal.xlsx
+++ b/app/templates/OT/OT-MUESTRAS/OT-MUESTRAS-Geofal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\OT\OT-SU-Y-AG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\OT\OT-MUESTRAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E29017-F877-4039-A481-83F46DF974D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D21D1E6-40FA-4350-8633-AA74E809FBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1536" windowWidth="23040" windowHeight="10920" xr2:uid="{7CAA3784-AC6A-4491-9DAE-0EC89CC1DDD5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7CAA3784-AC6A-4491-9DAE-0EC89CC1DDD5}"/>
   </bookViews>
   <sheets>
     <sheet name="HOJA 1 (2)" sheetId="3" r:id="rId1"/>
@@ -187,9 +187,6 @@
     <t>ASTM D2630</t>
   </si>
   <si>
-    <t>F-LEM-P-02.03</t>
-  </si>
-  <si>
     <t>BETZABETH SARAVIA</t>
   </si>
   <si>
@@ -197,6 +194,9 @@
   </si>
   <si>
     <t xml:space="preserve">OT DESIGADA A:    </t>
+  </si>
+  <si>
+    <t>F-LEM-P-02.01</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1060,7 @@
         <v>1</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -1075,7 +1075,7 @@
         <v>2</v>
       </c>
       <c r="I2" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -1569,7 +1569,7 @@
     </row>
     <row r="33" spans="1:9" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B33" s="48"/>
       <c r="C33" s="48"/>
@@ -1601,11 +1601,11 @@
       <c r="B36" s="45"/>
       <c r="C36" s="45"/>
       <c r="D36" s="46" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E36" s="46"/>
       <c r="F36" s="45" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G36" s="45"/>
       <c r="H36" s="45"/>

</xml_diff>